<commit_message>
fix(medicines): fix bug in function import vs sale with unit
</commit_message>
<xml_diff>
--- a/sample-medicines-import.xlsx
+++ b/sample-medicines-import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:U25"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -453,7 +453,7 @@
         <v>Giá bán</v>
       </c>
       <c r="K1" t="str">
-        <v>Thời hạn sử dụng (tháng)</v>
+        <v>Thời hạn sử dụng (ngày)</v>
       </c>
       <c r="L1" t="str">
         <v>Thành phần</v>
@@ -481,6 +481,9 @@
       </c>
       <c r="T1" t="str">
         <v>Thông tin khác</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Thời hạn sử dụng (tháng)</v>
       </c>
     </row>
     <row r="2">
@@ -515,7 +518,7 @@
         <v>6000</v>
       </c>
       <c r="K2">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L2" t="str">
         <v>Paracetamol 500mg</v>
@@ -576,9 +579,6 @@
       <c r="J3">
         <v>8000</v>
       </c>
-      <c r="K3">
-        <v>24</v>
-      </c>
       <c r="L3" t="str">
         <v>Amoxicillin trihydrate 250mg</v>
       </c>
@@ -605,6 +605,9 @@
       </c>
       <c r="T3" t="str">
         <v>Uống đủ liệu trình, không tự ý ngừng thuốc</v>
+      </c>
+      <c r="U3">
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -639,7 +642,7 @@
         <v>9500</v>
       </c>
       <c r="K4">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L4" t="str">
         <v>Ibuprofen 400mg</v>
@@ -700,9 +703,6 @@
       <c r="J5">
         <v>20000</v>
       </c>
-      <c r="K5">
-        <v>24</v>
-      </c>
       <c r="L5" t="str">
         <v>Cefuroxime axetil 250mg</v>
       </c>
@@ -729,6 +729,9 @@
       </c>
       <c r="T5" t="str">
         <v>Uống đủ liệu trình theo chỉ định của bác sĩ</v>
+      </c>
+      <c r="U5">
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -763,7 +766,7 @@
         <v>14000</v>
       </c>
       <c r="K6">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L6" t="str">
         <v>Omeprazole 20mg</v>
@@ -825,7 +828,7 @@
         <v>5500</v>
       </c>
       <c r="K7">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L7" t="str">
         <v>Metformin hydrochloride 500mg</v>
@@ -887,7 +890,7 @@
         <v>11000</v>
       </c>
       <c r="K8">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L8" t="str">
         <v>Amlodipine besylate 5mg</v>
@@ -949,7 +952,7 @@
         <v>25000</v>
       </c>
       <c r="K9">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L9" t="str">
         <v>Atorvastatin calcium 20mg</v>
@@ -1011,7 +1014,7 @@
         <v>12000</v>
       </c>
       <c r="K10">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L10" t="str">
         <v>Losartan potassium 50mg</v>
@@ -1073,7 +1076,7 @@
         <v>9000</v>
       </c>
       <c r="K11">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L11" t="str">
         <v>Levothyroxine sodium 100mcg</v>
@@ -1135,7 +1138,7 @@
         <v>7500</v>
       </c>
       <c r="K12">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L12" t="str">
         <v>Atenolol 50mg</v>
@@ -1197,7 +1200,7 @@
         <v>4000</v>
       </c>
       <c r="K13">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L13" t="str">
         <v>Furosemide 40mg</v>
@@ -1259,7 +1262,7 @@
         <v>6000</v>
       </c>
       <c r="K14">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L14" t="str">
         <v>Warfarin sodium 5mg</v>
@@ -1321,7 +1324,7 @@
         <v>3000</v>
       </c>
       <c r="K15">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L15" t="str">
         <v>Acetylsalicylic acid 100mg</v>
@@ -1382,9 +1385,6 @@
       <c r="J16">
         <v>15000</v>
       </c>
-      <c r="K16">
-        <v>24</v>
-      </c>
       <c r="L16" t="str">
         <v>Ciprofloxacin hydrochloride 500mg</v>
       </c>
@@ -1411,6 +1411,9 @@
       </c>
       <c r="T16" t="str">
         <v>Tránh ánh sáng mặt trời, uống đủ nước, không dùng với sữa</v>
+      </c>
+      <c r="U16">
+        <v>24</v>
       </c>
     </row>
     <row r="17">
@@ -1445,7 +1448,7 @@
         <v>11000</v>
       </c>
       <c r="K17">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L17" t="str">
         <v>Doxycycline hyclate 100mg</v>
@@ -1507,7 +1510,7 @@
         <v>7500</v>
       </c>
       <c r="K18">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L18" t="str">
         <v>Metronidazole 250mg</v>
@@ -1568,9 +1571,6 @@
       <c r="J19">
         <v>18000</v>
       </c>
-      <c r="K19">
-        <v>24</v>
-      </c>
       <c r="L19" t="str">
         <v>Clarithromycin 250mg</v>
       </c>
@@ -1597,6 +1597,9 @@
       </c>
       <c r="T19" t="str">
         <v>Uống đủ liệu trình, thận trọng với bệnh nhân có bệnh tim</v>
+      </c>
+      <c r="U19">
+        <v>24</v>
       </c>
     </row>
     <row r="20">
@@ -1630,9 +1633,6 @@
       <c r="J20">
         <v>22000</v>
       </c>
-      <c r="K20">
-        <v>24</v>
-      </c>
       <c r="L20" t="str">
         <v>Azithromycin dihydrate 500mg</v>
       </c>
@@ -1659,6 +1659,9 @@
       </c>
       <c r="T20" t="str">
         <v>Uống đủ liệu trình, thận trọng với bệnh nhân có bệnh tim</v>
+      </c>
+      <c r="U20">
+        <v>24</v>
       </c>
     </row>
     <row r="21">
@@ -1693,7 +1696,7 @@
         <v>16000</v>
       </c>
       <c r="K21">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L21" t="str">
         <v>Pantoprazole sodium 40mg</v>
@@ -1754,9 +1757,6 @@
       <c r="J22">
         <v>4000</v>
       </c>
-      <c r="K22">
-        <v>24</v>
-      </c>
       <c r="L22" t="str">
         <v>Glucose, Natri clorid, Kali clorid, Natri citrat</v>
       </c>
@@ -1783,6 +1783,9 @@
       </c>
       <c r="T22" t="str">
         <v>Bảo quản nơi khô ráo, tránh ẩm</v>
+      </c>
+      <c r="U22">
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -1817,7 +1820,7 @@
         <v>80000</v>
       </c>
       <c r="K23">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L23" t="str">
         <v>Chiết xuất lá thường xuân</v>
@@ -1878,9 +1881,6 @@
       <c r="J24">
         <v>25000</v>
       </c>
-      <c r="K24">
-        <v>24</v>
-      </c>
       <c r="L24" t="str">
         <v>Epinephrine 1mg/ml</v>
       </c>
@@ -1907,6 +1907,9 @@
       </c>
       <c r="T24" t="str">
         <v>Bảo quản ở nhiệt độ 2-8°C, tránh ánh sáng, chỉ dùng trong cấp cứu</v>
+      </c>
+      <c r="U24">
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -1941,7 +1944,7 @@
         <v>60000</v>
       </c>
       <c r="K25">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L25" t="str">
         <v>Acid fusidic 2%</v>
@@ -1973,7 +1976,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(medicines): fix bug in function import vs sale with unit (#60)
Co-authored-by: Nguyentung7193 <nguyentung260310@mail.com>
</commit_message>
<xml_diff>
--- a/sample-medicines-import.xlsx
+++ b/sample-medicines-import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:U25"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -453,7 +453,7 @@
         <v>Giá bán</v>
       </c>
       <c r="K1" t="str">
-        <v>Thời hạn sử dụng (tháng)</v>
+        <v>Thời hạn sử dụng (ngày)</v>
       </c>
       <c r="L1" t="str">
         <v>Thành phần</v>
@@ -481,6 +481,9 @@
       </c>
       <c r="T1" t="str">
         <v>Thông tin khác</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Thời hạn sử dụng (tháng)</v>
       </c>
     </row>
     <row r="2">
@@ -515,7 +518,7 @@
         <v>6000</v>
       </c>
       <c r="K2">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L2" t="str">
         <v>Paracetamol 500mg</v>
@@ -576,9 +579,6 @@
       <c r="J3">
         <v>8000</v>
       </c>
-      <c r="K3">
-        <v>24</v>
-      </c>
       <c r="L3" t="str">
         <v>Amoxicillin trihydrate 250mg</v>
       </c>
@@ -605,6 +605,9 @@
       </c>
       <c r="T3" t="str">
         <v>Uống đủ liệu trình, không tự ý ngừng thuốc</v>
+      </c>
+      <c r="U3">
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -639,7 +642,7 @@
         <v>9500</v>
       </c>
       <c r="K4">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L4" t="str">
         <v>Ibuprofen 400mg</v>
@@ -700,9 +703,6 @@
       <c r="J5">
         <v>20000</v>
       </c>
-      <c r="K5">
-        <v>24</v>
-      </c>
       <c r="L5" t="str">
         <v>Cefuroxime axetil 250mg</v>
       </c>
@@ -729,6 +729,9 @@
       </c>
       <c r="T5" t="str">
         <v>Uống đủ liệu trình theo chỉ định của bác sĩ</v>
+      </c>
+      <c r="U5">
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -763,7 +766,7 @@
         <v>14000</v>
       </c>
       <c r="K6">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L6" t="str">
         <v>Omeprazole 20mg</v>
@@ -825,7 +828,7 @@
         <v>5500</v>
       </c>
       <c r="K7">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L7" t="str">
         <v>Metformin hydrochloride 500mg</v>
@@ -887,7 +890,7 @@
         <v>11000</v>
       </c>
       <c r="K8">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L8" t="str">
         <v>Amlodipine besylate 5mg</v>
@@ -949,7 +952,7 @@
         <v>25000</v>
       </c>
       <c r="K9">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L9" t="str">
         <v>Atorvastatin calcium 20mg</v>
@@ -1011,7 +1014,7 @@
         <v>12000</v>
       </c>
       <c r="K10">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L10" t="str">
         <v>Losartan potassium 50mg</v>
@@ -1073,7 +1076,7 @@
         <v>9000</v>
       </c>
       <c r="K11">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L11" t="str">
         <v>Levothyroxine sodium 100mcg</v>
@@ -1135,7 +1138,7 @@
         <v>7500</v>
       </c>
       <c r="K12">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L12" t="str">
         <v>Atenolol 50mg</v>
@@ -1197,7 +1200,7 @@
         <v>4000</v>
       </c>
       <c r="K13">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L13" t="str">
         <v>Furosemide 40mg</v>
@@ -1259,7 +1262,7 @@
         <v>6000</v>
       </c>
       <c r="K14">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L14" t="str">
         <v>Warfarin sodium 5mg</v>
@@ -1321,7 +1324,7 @@
         <v>3000</v>
       </c>
       <c r="K15">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L15" t="str">
         <v>Acetylsalicylic acid 100mg</v>
@@ -1382,9 +1385,6 @@
       <c r="J16">
         <v>15000</v>
       </c>
-      <c r="K16">
-        <v>24</v>
-      </c>
       <c r="L16" t="str">
         <v>Ciprofloxacin hydrochloride 500mg</v>
       </c>
@@ -1411,6 +1411,9 @@
       </c>
       <c r="T16" t="str">
         <v>Tránh ánh sáng mặt trời, uống đủ nước, không dùng với sữa</v>
+      </c>
+      <c r="U16">
+        <v>24</v>
       </c>
     </row>
     <row r="17">
@@ -1445,7 +1448,7 @@
         <v>11000</v>
       </c>
       <c r="K17">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L17" t="str">
         <v>Doxycycline hyclate 100mg</v>
@@ -1507,7 +1510,7 @@
         <v>7500</v>
       </c>
       <c r="K18">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L18" t="str">
         <v>Metronidazole 250mg</v>
@@ -1568,9 +1571,6 @@
       <c r="J19">
         <v>18000</v>
       </c>
-      <c r="K19">
-        <v>24</v>
-      </c>
       <c r="L19" t="str">
         <v>Clarithromycin 250mg</v>
       </c>
@@ -1597,6 +1597,9 @@
       </c>
       <c r="T19" t="str">
         <v>Uống đủ liệu trình, thận trọng với bệnh nhân có bệnh tim</v>
+      </c>
+      <c r="U19">
+        <v>24</v>
       </c>
     </row>
     <row r="20">
@@ -1630,9 +1633,6 @@
       <c r="J20">
         <v>22000</v>
       </c>
-      <c r="K20">
-        <v>24</v>
-      </c>
       <c r="L20" t="str">
         <v>Azithromycin dihydrate 500mg</v>
       </c>
@@ -1659,6 +1659,9 @@
       </c>
       <c r="T20" t="str">
         <v>Uống đủ liệu trình, thận trọng với bệnh nhân có bệnh tim</v>
+      </c>
+      <c r="U20">
+        <v>24</v>
       </c>
     </row>
     <row r="21">
@@ -1693,7 +1696,7 @@
         <v>16000</v>
       </c>
       <c r="K21">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L21" t="str">
         <v>Pantoprazole sodium 40mg</v>
@@ -1754,9 +1757,6 @@
       <c r="J22">
         <v>4000</v>
       </c>
-      <c r="K22">
-        <v>24</v>
-      </c>
       <c r="L22" t="str">
         <v>Glucose, Natri clorid, Kali clorid, Natri citrat</v>
       </c>
@@ -1783,6 +1783,9 @@
       </c>
       <c r="T22" t="str">
         <v>Bảo quản nơi khô ráo, tránh ẩm</v>
+      </c>
+      <c r="U22">
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -1817,7 +1820,7 @@
         <v>80000</v>
       </c>
       <c r="K23">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L23" t="str">
         <v>Chiết xuất lá thường xuân</v>
@@ -1878,9 +1881,6 @@
       <c r="J24">
         <v>25000</v>
       </c>
-      <c r="K24">
-        <v>24</v>
-      </c>
       <c r="L24" t="str">
         <v>Epinephrine 1mg/ml</v>
       </c>
@@ -1907,6 +1907,9 @@
       </c>
       <c r="T24" t="str">
         <v>Bảo quản ở nhiệt độ 2-8°C, tránh ánh sáng, chỉ dùng trong cấp cứu</v>
+      </c>
+      <c r="U24">
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -1941,7 +1944,7 @@
         <v>60000</v>
       </c>
       <c r="K25">
-        <v>36</v>
+        <v>1080</v>
       </c>
       <c r="L25" t="str">
         <v>Acid fusidic 2%</v>
@@ -1973,7 +1976,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>